<commit_message>
added chapter 1 vocab
</commit_message>
<xml_diff>
--- a/worksheets/forms.xlsx
+++ b/worksheets/forms.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schmu\OneDrive\Desktop\Greek\NT Greek FC-git\worksheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schmu\source\repos\Greek\NT Greek FC-git\worksheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B03D240-18EF-41E1-8F64-B6A05C2EC000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC7718DB-9E51-4B9D-952F-77D239B6C73C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$F$29</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -262,10 +265,10 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -548,13 +551,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="13.7109375" customWidth="1"/>
-    <col min="4" max="4" width="3.140625" customWidth="1"/>
-    <col min="5" max="6" width="13.7109375" customWidth="1"/>
-    <col min="8" max="10" width="13.7109375" customWidth="1"/>
+    <col min="4" max="4" width="0.7109375" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" customWidth="1"/>
+    <col min="10" max="10" width="11.7109375" customWidth="1"/>
     <col min="12" max="12" width="11.5703125" customWidth="1"/>
     <col min="13" max="13" width="12.28515625" customWidth="1"/>
     <col min="14" max="14" width="13.140625" customWidth="1"/>
@@ -564,20 +570,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="14"/>
+      <c r="C1" s="13"/>
       <c r="D1" s="5"/>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="F1" s="14"/>
+      <c r="F1" s="13"/>
       <c r="G1" s="4"/>
-      <c r="I1" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="J1" s="14"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="4"/>
@@ -595,12 +597,6 @@
         <v>15</v>
       </c>
       <c r="G2" s="4"/>
-      <c r="I2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>15</v>
-      </c>
     </row>
     <row r="3" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -619,15 +615,6 @@
       <c r="F3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="4" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
@@ -640,15 +627,6 @@
         <v>4</v>
       </c>
       <c r="D4" s="1"/>
-      <c r="H4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>11</v>
-      </c>
     </row>
     <row r="5" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
@@ -661,35 +639,15 @@
         <v>5</v>
       </c>
       <c r="D5" s="1"/>
-      <c r="H5" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>12</v>
-      </c>
     </row>
     <row r="6" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H6" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="I6" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="J6" s="9" t="s">
-        <v>13</v>
-      </c>
       <c r="K6" s="10"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="14"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
+      <c r="C10" s="13"/>
     </row>
     <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
@@ -698,12 +656,6 @@
       <c r="C11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>39</v>
-      </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
@@ -715,15 +667,6 @@
       <c r="C12" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>40</v>
-      </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
@@ -735,15 +678,6 @@
       <c r="C13" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E13" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>41</v>
-      </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
@@ -755,15 +689,6 @@
       <c r="C14" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E14" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>42</v>
-      </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
@@ -776,26 +701,131 @@
         <v>32</v>
       </c>
       <c r="D15" s="10"/>
-      <c r="E15" s="11" t="s">
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B18" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="B22" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="C22" s="9" t="s">
         <v>43</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B24" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" s="13"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B25" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="B1:C1"/>
-    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B10:C10"/>
-    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="B24:C24"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="6" max="1048575" man="1"/>
   </colBreaks>

</xml_diff>